<commit_message>
Add new images: cocina.png and laverrap.png
</commit_message>
<xml_diff>
--- a/config_test.xlsx
+++ b/config_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\OneDrive\Escritorio\bio-quim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1434E8F9-8A03-42C5-ABAC-FB3E6D30274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF661068-849D-457F-A5C7-A7FCFE760970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,9 @@
     <sheet name="configuracion" sheetId="3" r:id="rId4"/>
     <sheet name="hero" sheetId="4" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Productos!$A$1:$K$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="77">
   <si>
     <t>images</t>
   </si>
@@ -153,21 +156,12 @@
     <t>Alcohol en Gel</t>
   </si>
   <si>
-    <t>Desengrasante</t>
-  </si>
-  <si>
     <t>Desodorante Pisos</t>
   </si>
   <si>
-    <t>Detergente Economico</t>
-  </si>
-  <si>
     <t>Detergente Super</t>
   </si>
   <si>
-    <t>Fajinador</t>
-  </si>
-  <si>
     <t>Jabon Para Manos</t>
   </si>
   <si>
@@ -256,6 +250,24 @@
   </si>
   <si>
     <t>Alcohol</t>
+  </si>
+  <si>
+    <t>Detergente Premium</t>
+  </si>
+  <si>
+    <t>Desinfectante Pisos</t>
+  </si>
+  <si>
+    <t>Envase x 500 ML</t>
+  </si>
+  <si>
+    <t>Envase x 250 ML</t>
+  </si>
+  <si>
+    <t>Desengrasante Cocina</t>
+  </si>
+  <si>
+    <t>Desengrasante Autos</t>
   </si>
 </sst>
 </file>
@@ -668,10 +680,10 @@
   <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="2" width="16.44140625" customWidth="1"/>
     <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.44140625" customWidth="1"/>
+    <col min="5" max="5" width="39.5546875" customWidth="1"/>
     <col min="6" max="6" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.5546875" customWidth="1"/>
     <col min="8" max="8" width="11.88671875" customWidth="1"/>
@@ -716,133 +728,129 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D2">
-        <v>30000</v>
+        <v>2100</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F2" s="7"/>
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D3">
-        <f>1250*5</f>
-        <v>6250</v>
+        <v>2100</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F3" s="7"/>
       <c r="H3" s="6"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" t="s">
         <v>47</v>
       </c>
-      <c r="B4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" t="s">
-        <v>53</v>
-      </c>
       <c r="D4">
-        <v>1250</v>
+        <v>3200</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="F4" s="7"/>
-      <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D5">
-        <f>1250*5</f>
-        <v>6250</v>
+        <v>1200</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F5" s="7"/>
-      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D6">
-        <v>960</v>
+        <v>1900</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D7">
-        <v>1250</v>
+        <v>2000</v>
       </c>
       <c r="E7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D8">
-        <v>600</v>
+        <v>2600</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F8" s="7"/>
     </row>
@@ -851,345 +859,340 @@
         <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D9">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F9" s="7"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
         <v>48</v>
       </c>
       <c r="D10">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F10" s="7"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="D11">
-        <v>600</v>
+        <v>3600</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F11" s="7"/>
-      <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D12">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="D13">
-        <v>1850</v>
+        <v>7500</v>
       </c>
       <c r="E13" t="s">
         <v>64</v>
       </c>
       <c r="F13" s="7"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D14">
-        <v>1500</v>
+        <v>7500</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F14" s="7"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D15">
-        <v>1600</v>
+        <v>7500</v>
       </c>
       <c r="E15" t="s">
         <v>64</v>
       </c>
-      <c r="F15" s="7"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D16">
-        <v>9500</v>
+        <v>3500</v>
       </c>
       <c r="E16" t="s">
         <v>64</v>
       </c>
-      <c r="F16" s="7"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D17">
-        <f>+D6*5</f>
-        <v>4800</v>
+        <v>5500</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D18">
-        <f t="shared" ref="D18:D27" si="0">+D7*5</f>
-        <v>6250</v>
+        <v>7000</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D19">
-        <f t="shared" si="0"/>
-        <v>3000</v>
+        <v>9900</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>72</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D20">
-        <f t="shared" si="0"/>
-        <v>5500</v>
+        <v>3500</v>
       </c>
       <c r="E20" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C21" t="s">
         <v>48</v>
       </c>
       <c r="D21">
-        <f t="shared" si="0"/>
-        <v>6000</v>
+        <v>7000</v>
       </c>
       <c r="E21" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="D22">
-        <f t="shared" si="0"/>
-        <v>3000</v>
+        <v>14000</v>
       </c>
       <c r="E22" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D23">
-        <f t="shared" si="0"/>
-        <v>7500</v>
+        <v>7000</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C24" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="D24">
-        <f t="shared" si="0"/>
-        <v>9250</v>
+        <v>11000</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+      <c r="F24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D25">
-        <f t="shared" si="0"/>
-        <v>7500</v>
+        <v>53000</v>
       </c>
       <c r="E25" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>43</v>
       </c>
       <c r="B26" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C26" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D26">
-        <f t="shared" si="0"/>
-        <v>8000</v>
+        <v>5800</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B27" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D27">
-        <f t="shared" si="0"/>
-        <v>47500</v>
+        <v>3200</v>
       </c>
       <c r="E27" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K26">
+      <sortCondition ref="B1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1238,95 +1241,95 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1345,8 +1348,8 @@
     <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" customWidth="1"/>
+    <col min="9" max="9" width="8.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -1380,31 +1383,31 @@
     </row>
     <row r="2" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="H2" s="5">
         <v>541127444019</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>